<commit_message>
Add KMeans clustering to EV analysis notebook
Replace ev_analysis.ipynb with clustering.ipynb: UMAP projection plus
auto-k KMeans (silhouette-selected), arrival time as minutes, and
labeled income/employment encodings.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RTS_Public_File_data_dictionary.xlsx
+++ b/data/RTS_Public_File_data_dictionary.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Household"/>
@@ -4470,7 +4470,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
       <c r="A150" s="25" t="s">
         <v>22</v>
       </c>
@@ -4481,7 +4481,7 @@
         <v>781</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
       <c r="A151" s="22"/>
       <c r="B151" s="26">
         <v>8</v>
@@ -4490,7 +4490,7 @@
         <v>782</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
       <c r="A152" s="8"/>
       <c r="B152" s="9"/>
       <c r="C152" s="8"/>
@@ -4502,14 +4502,14 @@
       <c r="B153" s="12"/>
       <c r="C153" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A154" s="13"/>
       <c r="B154" s="14"/>
       <c r="C154" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A155" s="25" t="s">
         <v>4</v>
       </c>
@@ -4520,7 +4520,7 @@
         <v>784</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A156" s="19"/>
       <c r="B156" s="20" t="s">
         <v>7</v>
@@ -4529,7 +4529,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A157" s="19"/>
       <c r="B157" s="20" t="s">
         <v>9</v>
@@ -4538,7 +4538,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
       <c r="A158" s="25" t="s">
         <v>22</v>
       </c>
@@ -4549,7 +4549,7 @@
         <v>785</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
       <c r="A159" s="22"/>
       <c r="B159" s="26">
         <v>8</v>
@@ -4558,7 +4558,7 @@
         <v>786</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
       <c r="A160" s="8"/>
       <c r="B160" s="9"/>
       <c r="C160" s="8"/>
@@ -4570,14 +4570,14 @@
       <c r="B161" s="12"/>
       <c r="C161" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A162" s="13"/>
       <c r="B162" s="14"/>
       <c r="C162" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="31.5" customFormat="1" s="10">
       <c r="A163" s="25" t="s">
         <v>4</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>788</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A164" s="19"/>
       <c r="B164" s="20" t="s">
         <v>7</v>
@@ -4597,7 +4597,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A165" s="19"/>
       <c r="B165" s="20" t="s">
         <v>9</v>
@@ -4606,7 +4606,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
       <c r="A166" s="25" t="s">
         <v>22</v>
       </c>
@@ -4617,7 +4617,7 @@
         <v>789</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
       <c r="A167" s="22"/>
       <c r="B167" s="26">
         <v>8</v>
@@ -4626,7 +4626,7 @@
         <v>790</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
       <c r="A168" s="8"/>
       <c r="B168" s="9"/>
       <c r="C168" s="8"/>
@@ -4638,14 +4638,14 @@
       <c r="B169" s="12"/>
       <c r="C169" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A170" s="13"/>
       <c r="B170" s="14"/>
       <c r="C170" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A171" s="16" t="s">
         <v>4</v>
       </c>
@@ -4656,7 +4656,7 @@
         <v>792</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A172" s="19"/>
       <c r="B172" s="20" t="s">
         <v>7</v>
@@ -4665,7 +4665,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A173" s="19"/>
       <c r="B173" s="20" t="s">
         <v>9</v>
@@ -4674,7 +4674,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
       <c r="A174" s="25" t="s">
         <v>22</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>411</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
       <c r="A175" s="22"/>
       <c r="B175" s="26">
         <v>8</v>
@@ -4694,7 +4694,7 @@
         <v>412</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
       <c r="A176" s="8"/>
       <c r="B176" s="9"/>
       <c r="C176" s="8"/>
@@ -4706,14 +4706,14 @@
       <c r="B177" s="12"/>
       <c r="C177" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A178" s="13"/>
       <c r="B178" s="14"/>
       <c r="C178" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A179" s="16" t="s">
         <v>4</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>794</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A180" s="19"/>
       <c r="B180" s="20" t="s">
         <v>7</v>
@@ -4733,7 +4733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A181" s="19"/>
       <c r="B181" s="20" t="s">
         <v>9</v>
@@ -4742,7 +4742,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
       <c r="A182" s="25" t="s">
         <v>22</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>795</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
       <c r="A183" s="22"/>
       <c r="B183" s="26">
         <v>8</v>
@@ -4762,7 +4762,7 @@
         <v>796</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
       <c r="A184" s="8"/>
       <c r="B184" s="9"/>
       <c r="C184" s="8"/>

</xml_diff>

<commit_message>
Add EV profile generation
</commit_message>
<xml_diff>
--- a/data/RTS_Public_File_data_dictionary.xlsx
+++ b/data/RTS_Public_File_data_dictionary.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Household"/>
@@ -4774,14 +4774,14 @@
       <c r="B185" s="12"/>
       <c r="C185" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A186" s="13"/>
       <c r="B186" s="14"/>
       <c r="C186" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A187" s="16" t="s">
         <v>4</v>
       </c>
@@ -4792,7 +4792,7 @@
         <v>798</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A188" s="19"/>
       <c r="B188" s="20" t="s">
         <v>7</v>
@@ -4801,7 +4801,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A189" s="19"/>
       <c r="B189" s="20" t="s">
         <v>9</v>
@@ -4810,7 +4810,7 @@
         <v>101</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
       <c r="A190" s="25" t="s">
         <v>22</v>
       </c>
@@ -4821,7 +4821,7 @@
         <v>799</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
       <c r="A191" s="19"/>
       <c r="B191" s="9">
         <v>5</v>
@@ -4830,7 +4830,7 @@
         <v>800</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
       <c r="A192" s="22" t="s">
         <v>37</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
       <c r="A193" s="19"/>
       <c r="B193" s="9"/>
       <c r="C193" s="21"/>
@@ -4853,14 +4853,14 @@
       <c r="B194" s="12"/>
       <c r="C194" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A195" s="13"/>
       <c r="B195" s="14"/>
       <c r="C195" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A196" s="16" t="s">
         <v>4</v>
       </c>
@@ -4871,7 +4871,7 @@
         <v>802</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A197" s="19"/>
       <c r="B197" s="20" t="s">
         <v>7</v>
@@ -4880,7 +4880,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A198" s="19"/>
       <c r="B198" s="20" t="s">
         <v>9</v>
@@ -4889,7 +4889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
       <c r="A199" s="25" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Add work-context fields to Profile
Add student_status, workplace_ev_charging, and workplace_loc.
Refactor work_arrangement to mark at-home workplaces as remote.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RTS_Public_File_data_dictionary.xlsx
+++ b/data/RTS_Public_File_data_dictionary.xlsx
@@ -7082,7 +7082,7 @@
       <c r="E85" s="45"/>
       <c r="F85" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
       <c r="A86" s="19"/>
       <c r="B86" s="9">
         <v>2</v>
@@ -7094,7 +7094,7 @@
       <c r="E86" s="45"/>
       <c r="F86" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
       <c r="A87" s="22" t="s">
         <v>37</v>
       </c>
@@ -7108,7 +7108,7 @@
       <c r="E87" s="45"/>
       <c r="F87" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
       <c r="A88" s="19"/>
       <c r="B88" s="9"/>
       <c r="C88" s="21"/>
@@ -7116,7 +7116,7 @@
       <c r="E88" s="45"/>
       <c r="F88" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A89" s="11" t="s">
         <v>483</v>
       </c>
@@ -7126,7 +7126,7 @@
       <c r="E89" s="45"/>
       <c r="F89" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A90" s="13"/>
       <c r="B90" s="14"/>
       <c r="C90" s="15" t="s">
@@ -7136,7 +7136,7 @@
       <c r="E90" s="45"/>
       <c r="F90" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A91" s="16" t="s">
         <v>4</v>
       </c>
@@ -7150,7 +7150,7 @@
       <c r="E91" s="45"/>
       <c r="F91" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A92" s="19"/>
       <c r="B92" s="20" t="s">
         <v>7</v>
@@ -7162,7 +7162,7 @@
       <c r="E92" s="45"/>
       <c r="F92" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A93" s="19"/>
       <c r="B93" s="20" t="s">
         <v>9</v>
@@ -7174,7 +7174,7 @@
       <c r="E93" s="45"/>
       <c r="F93" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="25" t="s">
         <v>22</v>
       </c>
@@ -7188,7 +7188,7 @@
       <c r="E94" s="45"/>
       <c r="F94" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="19"/>
       <c r="B95" s="9">
         <v>2</v>
@@ -7200,7 +7200,7 @@
       <c r="E95" s="45"/>
       <c r="F95" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="19"/>
       <c r="B96" s="9">
         <v>998</v>
@@ -7212,7 +7212,7 @@
       <c r="E96" s="45"/>
       <c r="F96" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="22" t="s">
         <v>37</v>
       </c>
@@ -7226,7 +7226,7 @@
       <c r="E97" s="45"/>
       <c r="F97" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="19"/>
       <c r="B98" s="9"/>
       <c r="C98" s="21"/>
@@ -7234,7 +7234,7 @@
       <c r="E98" s="45"/>
       <c r="F98" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A99" s="11" t="s">
         <v>485</v>
       </c>
@@ -7244,7 +7244,7 @@
       <c r="E99" s="45"/>
       <c r="F99" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A100" s="13"/>
       <c r="B100" s="14"/>
       <c r="C100" s="15" t="s">
@@ -7254,7 +7254,7 @@
       <c r="E100" s="45"/>
       <c r="F100" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A101" s="16" t="s">
         <v>4</v>
       </c>
@@ -7268,7 +7268,7 @@
       <c r="E101" s="45"/>
       <c r="F101" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A102" s="19"/>
       <c r="B102" s="20" t="s">
         <v>7</v>
@@ -7280,7 +7280,7 @@
       <c r="E102" s="45"/>
       <c r="F102" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A103" s="19"/>
       <c r="B103" s="20" t="s">
         <v>9</v>
@@ -7292,7 +7292,7 @@
       <c r="E103" s="45"/>
       <c r="F103" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
       <c r="A104" s="25" t="s">
         <v>22</v>
       </c>
@@ -7306,7 +7306,7 @@
       <c r="E104" s="45"/>
       <c r="F104" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
       <c r="A105" s="19"/>
       <c r="B105" s="9">
         <v>2</v>
@@ -7318,7 +7318,7 @@
       <c r="E105" s="45"/>
       <c r="F105" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
       <c r="A106" s="22" t="s">
         <v>37</v>
       </c>
@@ -7332,7 +7332,7 @@
       <c r="E106" s="45"/>
       <c r="F106" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
       <c r="A107" s="8"/>
       <c r="B107" s="9"/>
       <c r="C107" s="8"/>
@@ -7340,7 +7340,7 @@
       <c r="E107" s="45"/>
       <c r="F107" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A108" s="11" t="s">
         <v>487</v>
       </c>
@@ -7350,7 +7350,7 @@
       <c r="E108" s="45"/>
       <c r="F108" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A109" s="13"/>
       <c r="B109" s="14"/>
       <c r="C109" s="15" t="s">
@@ -7360,7 +7360,7 @@
       <c r="E109" s="45"/>
       <c r="F109" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="32.25" customFormat="1" s="10">
       <c r="A110" s="16" t="s">
         <v>4</v>
       </c>
@@ -7374,7 +7374,7 @@
       <c r="E110" s="45"/>
       <c r="F110" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A111" s="19"/>
       <c r="B111" s="20" t="s">
         <v>7</v>
@@ -7386,7 +7386,7 @@
       <c r="E111" s="45"/>
       <c r="F111" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A112" s="19"/>
       <c r="B112" s="20" t="s">
         <v>9</v>
@@ -7398,7 +7398,7 @@
       <c r="E112" s="45"/>
       <c r="F112" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="25" t="s">
         <v>22</v>
       </c>
@@ -7412,7 +7412,7 @@
       <c r="E113" s="45"/>
       <c r="F113" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="19"/>
       <c r="B114" s="9">
         <v>2</v>
@@ -7424,7 +7424,7 @@
       <c r="E114" s="45"/>
       <c r="F114" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
       <c r="A115" s="22" t="s">
         <v>37</v>
       </c>
@@ -7438,7 +7438,7 @@
       <c r="E115" s="45"/>
       <c r="F115" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
       <c r="A116" s="8"/>
       <c r="B116" s="9"/>
       <c r="C116" s="8"/>

</xml_diff>

<commit_message>
Generalize profile generation and add demographic + trip context fields
Drop EV-only household filter so profiles cover all licensed drivers with
trips. Add per-trip vehicle linkage via MODE_HH_VEHICLE -> VEHNUM, plus
new Profile fields (home_type, home_ownership, day_of_week, household_size,
gender, race_ethnicity) and new Trip fields (travelers_total, travel_mode)
to support demographics x mobility analysis.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RTS_Public_File_data_dictionary.xlsx
+++ b/data/RTS_Public_File_data_dictionary.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Household"/>
@@ -7968,7 +7968,7 @@
       <c r="E160" s="45"/>
       <c r="F160" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="33">
       <c r="A161" s="19"/>
       <c r="B161" s="9">
         <v>6</v>
@@ -7980,7 +7980,7 @@
       <c r="E161" s="45"/>
       <c r="F161" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="19.5">
       <c r="A162" s="22" t="s">
         <v>37</v>
       </c>
@@ -7994,7 +7994,7 @@
       <c r="E162" s="45"/>
       <c r="F162" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="19.5">
       <c r="A163" s="8"/>
       <c r="B163" s="9"/>
       <c r="C163" s="8"/>
@@ -8002,7 +8002,7 @@
       <c r="E163" s="45"/>
       <c r="F163" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A164" s="11" t="s">
         <v>509</v>
       </c>
@@ -8012,7 +8012,7 @@
       <c r="E164" s="45"/>
       <c r="F164" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A165" s="13"/>
       <c r="B165" s="14"/>
       <c r="C165" s="15" t="s">
@@ -8022,7 +8022,7 @@
       <c r="E165" s="45"/>
       <c r="F165" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="33.75" customFormat="1" s="10">
       <c r="A166" s="16" t="s">
         <v>4</v>
       </c>
@@ -8036,7 +8036,7 @@
       <c r="E166" s="45"/>
       <c r="F166" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A167" s="19"/>
       <c r="B167" s="20" t="s">
         <v>7</v>
@@ -8048,7 +8048,7 @@
       <c r="E167" s="45"/>
       <c r="F167" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A168" s="19"/>
       <c r="B168" s="20" t="s">
         <v>9</v>
@@ -8060,7 +8060,7 @@
       <c r="E168" s="45"/>
       <c r="F168" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
       <c r="A169" s="25" t="s">
         <v>22</v>
       </c>
@@ -8074,7 +8074,7 @@
       <c r="E169" s="45"/>
       <c r="F169" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
       <c r="A170" s="19"/>
       <c r="B170" s="9">
         <v>5</v>
@@ -8086,7 +8086,7 @@
       <c r="E170" s="45"/>
       <c r="F170" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
       <c r="A171" s="22" t="s">
         <v>37</v>
       </c>
@@ -8100,7 +8100,7 @@
       <c r="E171" s="45"/>
       <c r="F171" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="8"/>
       <c r="B172" s="9"/>
       <c r="C172" s="8"/>
@@ -8108,7 +8108,7 @@
       <c r="E172" s="45"/>
       <c r="F172" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A173" s="11" t="s">
         <v>513</v>
       </c>
@@ -8118,7 +8118,7 @@
       <c r="E173" s="45"/>
       <c r="F173" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A174" s="13"/>
       <c r="B174" s="14"/>
       <c r="C174" s="15" t="s">
@@ -8128,7 +8128,7 @@
       <c r="E174" s="45"/>
       <c r="F174" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="20.25" customFormat="1" s="10">
       <c r="A175" s="16" t="s">
         <v>4</v>
       </c>
@@ -8142,7 +8142,7 @@
       <c r="E175" s="45"/>
       <c r="F175" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A176" s="19"/>
       <c r="B176" s="20" t="s">
         <v>7</v>
@@ -8154,7 +8154,7 @@
       <c r="E176" s="45"/>
       <c r="F176" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A177" s="19"/>
       <c r="B177" s="20" t="s">
         <v>9</v>
@@ -8166,7 +8166,7 @@
       <c r="E177" s="45"/>
       <c r="F177" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
       <c r="A178" s="25" t="s">
         <v>22</v>
       </c>
@@ -8180,7 +8180,7 @@
       <c r="E178" s="45"/>
       <c r="F178" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
       <c r="A179" s="19"/>
       <c r="B179" s="9">
         <v>2</v>
@@ -8192,7 +8192,7 @@
       <c r="E179" s="45"/>
       <c r="F179" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
       <c r="A180" s="19"/>
       <c r="B180" s="9">
         <v>3</v>
@@ -8204,7 +8204,7 @@
       <c r="E180" s="45"/>
       <c r="F180" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
       <c r="A181" s="19"/>
       <c r="B181" s="9">
         <v>4</v>
@@ -8216,7 +8216,7 @@
       <c r="E181" s="45"/>
       <c r="F181" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="33">
       <c r="A182" s="19"/>
       <c r="B182" s="9">
         <v>5</v>
@@ -8228,7 +8228,7 @@
       <c r="E182" s="45"/>
       <c r="F182" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
       <c r="A183" s="19"/>
       <c r="B183" s="9">
         <v>6</v>
@@ -8240,7 +8240,7 @@
       <c r="E183" s="45"/>
       <c r="F183" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5">
       <c r="A184" s="22" t="s">
         <v>37</v>
       </c>
@@ -8254,7 +8254,7 @@
       <c r="E184" s="45"/>
       <c r="F184" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
       <c r="A185" s="8"/>
       <c r="B185" s="9"/>
       <c r="C185" s="8"/>
@@ -8262,7 +8262,7 @@
       <c r="E185" s="45"/>
       <c r="F185" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A186" s="11" t="s">
         <v>521</v>
       </c>
@@ -8272,7 +8272,7 @@
       <c r="E186" s="45"/>
       <c r="F186" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A187" s="13"/>
       <c r="B187" s="14"/>
       <c r="C187" s="15" t="s">
@@ -8282,7 +8282,7 @@
       <c r="E187" s="45"/>
       <c r="F187" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="20.25" customFormat="1" s="10">
       <c r="A188" s="16" t="s">
         <v>4</v>
       </c>
@@ -8296,7 +8296,7 @@
       <c r="E188" s="45"/>
       <c r="F188" s="45"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A189" s="19"/>
       <c r="B189" s="20" t="s">
         <v>7</v>
@@ -16906,7 +16906,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A163" s="19"/>
       <c r="B163" s="20">
         <v>18</v>

</xml_diff>

<commit_message>
Count PHEV as EV; add cluster radars; regen filtered artifact
- profiles_to_df flags has_ev for both Electric and Plug-in Hybrid
- clustering notebook: add per-cluster radar grid (commute intensity,
  trip portfolio, life stage) after graph_cluster panels
- filter_profiles: re-enable artifact write at threshold 0.8 to refresh
  filtered_profiles.json under new PHEV-inclusive has_ev semantics
- profile_validation notebook: regenerated outputs against refreshed
  filtered_profiles.json

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RTS_Public_File_data_dictionary.xlsx
+++ b/data/RTS_Public_File_data_dictionary.xlsx
@@ -16888,7 +16888,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A161" s="19"/>
       <c r="B161" s="20">
         <v>16</v>
@@ -16897,7 +16897,7 @@
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A162" s="19"/>
       <c r="B162" s="20">
         <v>17</v>
@@ -16906,7 +16906,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A163" s="19"/>
       <c r="B163" s="20">
         <v>18</v>
@@ -16915,7 +16915,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A164" s="19"/>
       <c r="B164" s="20">
         <v>77</v>
@@ -16924,7 +16924,7 @@
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A165" s="19"/>
       <c r="B165" s="20">
         <v>99</v>
@@ -16933,7 +16933,7 @@
         <v>36</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="19.5">
       <c r="A166" s="22" t="s">
         <v>37</v>
       </c>
@@ -16944,26 +16944,26 @@
         <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="19.5">
       <c r="A167" s="19"/>
       <c r="B167" s="9"/>
       <c r="C167" s="21"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75" customFormat="1" s="10">
       <c r="A168" s="11" t="s">
         <v>86</v>
       </c>
       <c r="B168" s="12"/>
       <c r="C168" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="20.25" customFormat="1" s="10">
       <c r="A169" s="13"/>
       <c r="B169" s="14"/>
       <c r="C169" s="15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="20.25" customFormat="1" s="10">
       <c r="A170" s="25" t="s">
         <v>4</v>
       </c>
@@ -16974,7 +16974,7 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A171" s="19"/>
       <c r="B171" s="20" t="s">
         <v>7</v>
@@ -16983,7 +16983,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A172" s="19"/>
       <c r="B172" s="20" t="s">
         <v>9</v>
@@ -16992,7 +16992,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A173" s="19" t="s">
         <v>22</v>
       </c>
@@ -17003,7 +17003,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A174" s="19"/>
       <c r="B174" s="20">
         <v>2</v>
@@ -17012,7 +17012,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A175" s="19"/>
       <c r="B175" s="20">
         <v>3</v>
@@ -17021,7 +17021,7 @@
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A176" s="19"/>
       <c r="B176" s="20">
         <v>4</v>
@@ -17030,7 +17030,7 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A177" s="19"/>
       <c r="B177" s="20">
         <v>5</v>
@@ -17039,7 +17039,7 @@
         <v>42</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A178" s="19"/>
       <c r="B178" s="20">
         <v>6</v>
@@ -17048,7 +17048,7 @@
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A179" s="19"/>
       <c r="B179" s="20">
         <v>7</v>
@@ -17057,7 +17057,7 @@
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A180" s="19"/>
       <c r="B180" s="20">
         <v>8</v>
@@ -17066,7 +17066,7 @@
         <v>45</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A181" s="19"/>
       <c r="B181" s="20">
         <v>9</v>
@@ -17075,7 +17075,7 @@
         <v>46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A182" s="19"/>
       <c r="B182" s="20">
         <v>10</v>
@@ -17084,7 +17084,7 @@
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A183" s="19"/>
       <c r="B183" s="20">
         <v>11</v>
@@ -17093,7 +17093,7 @@
         <v>48</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A184" s="19"/>
       <c r="B184" s="20">
         <v>12</v>
@@ -17102,7 +17102,7 @@
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A185" s="19"/>
       <c r="B185" s="20">
         <v>13</v>
@@ -17111,7 +17111,7 @@
         <v>50</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A186" s="19"/>
       <c r="B186" s="20">
         <v>14</v>
@@ -17120,7 +17120,7 @@
         <v>51</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A187" s="19"/>
       <c r="B187" s="20">
         <v>15</v>
@@ -17129,7 +17129,7 @@
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A188" s="19"/>
       <c r="B188" s="20">
         <v>16</v>
@@ -17138,7 +17138,7 @@
         <v>53</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75" customFormat="1" s="10">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5" customFormat="1" s="10">
       <c r="A189" s="19"/>
       <c r="B189" s="20">
         <v>18</v>
@@ -17147,7 +17147,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
       <c r="A190" s="22" t="s">
         <v>37</v>
       </c>

</xml_diff>